<commit_message>
Update Stasjonspunktlighet og antall avganger Telemark fylkeskommune.xlsx
</commit_message>
<xml_diff>
--- a/Data/Mobilitet_i_Telemark/Jernbane/Punktlighet/Måned/Stasjonspunktlighet og antall avganger Telemark fylkeskommune.xlsx
+++ b/Data/Mobilitet_i_Telemark/Jernbane/Punktlighet/Måned/Stasjonspunktlighet og antall avganger Telemark fylkeskommune.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://telemarkfylke-my.sharepoint.com/personal/kjell-tore_haustveit_telemarkfylke_no/Documents/GitHub/Telemark/Data/Mobilitet_i_Telemark/Jernbane/Punktlighet/Måned/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADA43858-8B26-44BF-A7EC-41294D8417BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{ADA43858-8B26-44BF-A7EC-41294D8417BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACF8F83A-1B56-4766-A13C-99D8B980294A}"/>
   <bookViews>
-    <workbookView xWindow="3516" yWindow="552" windowWidth="26940" windowHeight="15588" xr2:uid="{2D5B676A-325C-4B2C-A14A-0D70DC3CBF00}"/>
+    <workbookView xWindow="28980" yWindow="972" windowWidth="26940" windowHeight="15588" xr2:uid="{2D5B676A-325C-4B2C-A14A-0D70DC3CBF00}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1B7AEA9-921D-4B91-9F31-E3C4A8CF7380}">
-  <dimension ref="A1:J798"/>
+  <dimension ref="A1:H800"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
@@ -748,7 +748,7 @@
     <col min="25" max="25" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>78</v>
       </c>
@@ -773,11 +773,8 @@
       <c r="H1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="J1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -803,7 +800,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>88</v>
       </c>
@@ -829,7 +826,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>88</v>
       </c>
@@ -855,7 +852,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -881,7 +878,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>88</v>
       </c>
@@ -907,7 +904,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>88</v>
       </c>
@@ -933,7 +930,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>88</v>
       </c>
@@ -959,7 +956,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>88</v>
       </c>
@@ -985,7 +982,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>88</v>
       </c>
@@ -1011,7 +1008,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>88</v>
       </c>
@@ -1037,7 +1034,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>88</v>
       </c>
@@ -1063,7 +1060,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -1089,7 +1086,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>88</v>
       </c>
@@ -1115,7 +1112,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>88</v>
       </c>
@@ -1141,7 +1138,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>88</v>
       </c>
@@ -21497,6 +21494,11 @@
       </c>
       <c r="H798">
         <v>86</v>
+      </c>
+    </row>
+    <row r="800" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A800" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -21509,12 +21511,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="304c15a9-2ddf-417f-8912-8cf6a1609eab">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ec2c31f6-e4da-4ac2-b928-7a50ed07fae6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21779,20 +21783,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="304c15a9-2ddf-417f-8912-8cf6a1609eab">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ec2c31f6-e4da-4ac2-b928-7a50ed07fae6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC802BAF-90BE-44F6-9844-7FDCFB831856}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5609B1E5-D8AE-4DAD-8CA9-C6DA9FE08DBE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="304c15a9-2ddf-417f-8912-8cf6a1609eab"/>
+    <ds:schemaRef ds:uri="ec2c31f6-e4da-4ac2-b928-7a50ed07fae6"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -21817,12 +21822,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5609B1E5-D8AE-4DAD-8CA9-C6DA9FE08DBE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC802BAF-90BE-44F6-9844-7FDCFB831856}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="304c15a9-2ddf-417f-8912-8cf6a1609eab"/>
-    <ds:schemaRef ds:uri="ec2c31f6-e4da-4ac2-b928-7a50ed07fae6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>